<commit_message>
change the all workout .csc to xlxs
</commit_message>
<xml_diff>
--- a/Bro_Split.xlsx
+++ b/Bro_Split.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mostafa\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UNIVERSITY\GraduationProject\MoveOn.FastAPI\WorkoutGeneration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F334F847-2182-48F6-B056-0E358BE5EE63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A34B533F-27FC-40B4-9C86-2430E2AFAAC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,24 +19,11 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$A$181</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="953" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="953" uniqueCount="128">
   <si>
     <t>Muscle_Group</t>
   </si>
@@ -399,9 +386,6 @@
   </si>
   <si>
     <t>Legs_Variation_5</t>
-  </si>
-  <si>
-    <t>Donkey Calf Raises</t>
   </si>
   <si>
     <t>Legs_Variation_6</t>
@@ -4180,7 +4164,7 @@
         <v>4</v>
       </c>
       <c r="D161" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E161" s="2" t="s">
         <v>16</v>
@@ -4220,7 +4204,7 @@
         <v>6</v>
       </c>
       <c r="D163" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E163" s="2" t="s">
         <v>9</v>
@@ -4340,7 +4324,7 @@
         <v>6</v>
       </c>
       <c r="D169" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E169" s="2" t="s">
         <v>9</v>
@@ -4400,7 +4384,7 @@
         <v>3</v>
       </c>
       <c r="D172" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E172" s="2" t="s">
         <v>16</v>
@@ -4580,7 +4564,7 @@
         <v>6</v>
       </c>
       <c r="D181" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E181" s="2" t="s">
         <v>16</v>
@@ -4651,7 +4635,7 @@
         <v>4</v>
       </c>
       <c r="D185" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E185" s="2" t="s">
         <v>16</v>
@@ -4696,13 +4680,13 @@
         <v>100</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C188" s="2">
         <v>1</v>
       </c>
       <c r="D188" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E188" s="2" t="s">
         <v>9</v>
@@ -4713,13 +4697,13 @@
         <v>100</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C189" s="2">
         <v>2</v>
       </c>
       <c r="D189" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E189" s="2" t="s">
         <v>9</v>
@@ -4730,7 +4714,7 @@
         <v>100</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C190" s="2">
         <v>3</v>
@@ -4747,7 +4731,7 @@
         <v>100</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C191" s="2">
         <v>4</v>
@@ -4764,7 +4748,7 @@
         <v>100</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C192" s="2">
         <v>5</v>
@@ -4781,13 +4765,13 @@
         <v>100</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C193" s="2">
         <v>6</v>
       </c>
       <c r="D193" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E193" s="2" t="s">
         <v>16</v>

</xml_diff>